<commit_message>
Final Project Plan Update
</commit_message>
<xml_diff>
--- a/docs/Project 2 Plan.xlsx
+++ b/docs/Project 2 Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57bb492ad5be0872/Desktop/School/CS-2430/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="249" documentId="8_{F9671BB7-C4F0-4247-ABF4-8FE418D4BC48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08A5445A-8D9B-4515-9419-6466EB63C29F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{A35F477B-69E0-4508-A779-2766FB3E9DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3072DF68-7313-4DFC-BC4F-F3A883A58564}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" firstSheet="1" activeTab="1" xr2:uid="{34D08FD4-51C7-4A98-AE26-ECA49DBE509F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="103">
   <si>
     <t>Group 2 Project 1: Set Operations</t>
   </si>
@@ -180,9 +180,6 @@
     <t>Individual</t>
   </si>
   <si>
-    <t>Incomplete</t>
-  </si>
-  <si>
     <t>Checkpoint</t>
   </si>
   <si>
@@ -325,6 +322,30 @@
   </si>
   <si>
     <t xml:space="preserve">    Screencast Brief Summary</t>
+  </si>
+  <si>
+    <t>Commit: 8dfb9ab2dbd0b928564f1b64efb2b5b00f3a7826</t>
+  </si>
+  <si>
+    <t>Commit: 1dfaf00be5cce80b0503e3197fed6785ad72c9cd</t>
+  </si>
+  <si>
+    <t>Commit: 97bd8cd7bc7709d04eaba924adf7d7da144f2d46</t>
+  </si>
+  <si>
+    <t>Commit: e498ba675921640d726b4f4e3584dc916b78c91a</t>
+  </si>
+  <si>
+    <t>Commit: cbee49782bce74e1aac0a84f2978de9e92ff2943</t>
+  </si>
+  <si>
+    <t>Commit: 3b5082e94c2c45e38a81edcc30bd1599c97cef68</t>
+  </si>
+  <si>
+    <t>Commit: db9f858b65b4748264e9546aa6c7957f68476f15</t>
+  </si>
+  <si>
+    <t>Commit: 2b8e3ceeb14ab68acd05f1a2cc19283b36dec617</t>
   </si>
 </sst>
 </file>
@@ -557,6 +578,7 @@
     <xf numFmtId="14" fontId="6" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -566,7 +588,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -1336,10 +1357,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1747,25 +1764,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
@@ -1845,37 +1862,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
@@ -1884,15 +1901,15 @@
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
@@ -1938,7 +1955,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>6</v>
@@ -1957,7 +1974,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>46</v>
@@ -1976,7 +1993,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>46</v>
@@ -1985,15 +2002,17 @@
         <v>46103</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E10" s="5">
+        <v>46103</v>
+      </c>
       <c r="F10" s="21"/>
       <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>20</v>
@@ -2002,15 +2021,17 @@
         <v>46103</v>
       </c>
       <c r="D11" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E11" s="5">
+        <v>46105</v>
+      </c>
       <c r="F11" s="21"/>
       <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>46</v>
@@ -2019,9 +2040,11 @@
         <v>46103</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E12" s="5">
+        <v>46103</v>
+      </c>
       <c r="F12" s="10"/>
       <c r="G12" s="4"/>
     </row>
@@ -2034,15 +2057,15 @@
       <c r="D14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A15" s="35" t="s">
+      <c r="A15" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
@@ -2069,7 +2092,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>20</v>
@@ -2088,7 +2111,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>20</v>
@@ -2107,7 +2130,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>6</v>
@@ -2141,12 +2164,12 @@
       </c>
       <c r="F20" s="10"/>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>20</v>
@@ -2161,13 +2184,13 @@
         <v>46090</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G21" s="4"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>8</v>
@@ -2183,12 +2206,12 @@
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>20</v>
@@ -2203,7 +2226,7 @@
         <v>46096</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G23" s="4"/>
     </row>
@@ -2237,15 +2260,19 @@
         <v>46097</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E25" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E25" s="5">
+        <v>46097</v>
+      </c>
       <c r="F25" s="10"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="4" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>4</v>
@@ -2254,15 +2281,19 @@
         <v>46102</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E26" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E26" s="5">
+        <v>46102</v>
+      </c>
       <c r="F26" s="10"/>
-      <c r="G26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>20</v>
@@ -2271,7 +2302,7 @@
         <v>46102</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="22"/>
@@ -2279,7 +2310,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>6</v>
@@ -2288,15 +2319,17 @@
         <v>46102</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E28" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E28" s="5">
+        <v>46105</v>
+      </c>
       <c r="F28" s="10"/>
       <c r="G28" s="4"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>8</v>
@@ -2305,15 +2338,17 @@
         <v>46102</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E29" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E29" s="5">
+        <v>46102</v>
+      </c>
       <c r="F29" s="10"/>
       <c r="G29" s="4"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>8</v>
@@ -2322,15 +2357,17 @@
         <v>46102</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E30" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E30" s="5">
+        <v>46102</v>
+      </c>
       <c r="F30" s="10"/>
       <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>4</v>
@@ -2339,15 +2376,17 @@
         <v>46102</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E31" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E31" s="5">
+        <v>46102</v>
+      </c>
       <c r="F31" s="10"/>
       <c r="G31" s="4"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>4</v>
@@ -2356,15 +2395,17 @@
         <v>46102</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E32" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E32" s="5">
+        <v>46102</v>
+      </c>
       <c r="F32" s="10"/>
       <c r="G32" s="4"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>20</v>
@@ -2373,9 +2414,11 @@
         <v>46102</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E33" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E33" s="5">
+        <v>46103</v>
+      </c>
       <c r="F33" s="10"/>
       <c r="G33" s="4"/>
     </row>
@@ -2390,9 +2433,11 @@
         <v>46102</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E34" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E34" s="5">
+        <v>46104</v>
+      </c>
       <c r="F34" s="10"/>
       <c r="G34" s="4"/>
     </row>
@@ -2407,9 +2452,11 @@
         <v>46102</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E35" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E35" s="5">
+        <v>46103</v>
+      </c>
       <c r="F35" s="10"/>
       <c r="G35" s="4"/>
     </row>
@@ -2424,24 +2471,26 @@
         <v>46102</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E36" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E36" s="5">
+        <v>46102</v>
+      </c>
       <c r="F36" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G36" s="4"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="35"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="35"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
@@ -2468,7 +2517,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>4</v>
@@ -2484,7 +2533,7 @@
       </c>
       <c r="F41" s="10"/>
       <c r="G41" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.4">
@@ -2524,7 +2573,7 @@
       </c>
       <c r="F43" s="10"/>
       <c r="G43" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.4">
@@ -2545,7 +2594,7 @@
       </c>
       <c r="F44" s="10"/>
       <c r="G44" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
@@ -2553,7 +2602,7 @@
         <v>24</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C45" s="7">
         <v>46089</v>
@@ -2569,7 +2618,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A46" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>4</v>
@@ -2585,12 +2634,12 @@
       </c>
       <c r="F46" s="10"/>
       <c r="G46" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>4</v>
@@ -2606,12 +2655,12 @@
       </c>
       <c r="F47" s="10"/>
       <c r="G47" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>6</v>
@@ -2627,12 +2676,12 @@
       </c>
       <c r="F48" s="10"/>
       <c r="G48" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A49" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>6</v>
@@ -2648,7 +2697,7 @@
       </c>
       <c r="F49" s="10"/>
       <c r="G49" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.4">
@@ -2669,12 +2718,12 @@
       </c>
       <c r="F50" s="10"/>
       <c r="G50" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A51" s="29" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B51" s="29" t="s">
         <v>8</v>
@@ -2685,17 +2734,17 @@
       <c r="D51" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="E51" s="38">
+      <c r="E51" s="35">
         <v>46092</v>
       </c>
       <c r="F51" s="28"/>
       <c r="G51" s="29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A52" s="31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B52" s="31" t="s">
         <v>4</v>
@@ -2711,7 +2760,7 @@
       </c>
       <c r="F52" s="30"/>
       <c r="G52" s="31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.4">
@@ -2744,11 +2793,15 @@
         <v>46103</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="E54" s="17"/>
+        <v>33</v>
+      </c>
+      <c r="E54" s="17">
+        <v>46103</v>
+      </c>
       <c r="F54" s="24"/>
-      <c r="G54" s="16"/>
+      <c r="G54" s="16" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A55" s="20"/>
@@ -2757,15 +2810,15 @@
       <c r="E55" s="3"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A57" s="35" t="s">
+      <c r="A57" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B57" s="35"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="35"/>
+      <c r="B57" s="36"/>
+      <c r="C57" s="36"/>
+      <c r="D57" s="36"/>
+      <c r="E57" s="36"/>
+      <c r="F57" s="36"/>
+      <c r="G57" s="36"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" s="2" t="s">
@@ -2801,15 +2854,19 @@
         <v>46102</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E59" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E59" s="5">
+        <v>46102</v>
+      </c>
       <c r="F59" s="10"/>
-      <c r="G59" s="4"/>
+      <c r="G59" s="4" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>8</v>
@@ -2818,15 +2875,19 @@
         <v>46102</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E60" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E60" s="5">
+        <v>46102</v>
+      </c>
       <c r="F60" s="10"/>
-      <c r="G60" s="4"/>
+      <c r="G60" s="4" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B61" s="4" t="s">
         <v>8</v>
@@ -2835,11 +2896,15 @@
         <v>46102</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E61" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E61" s="5">
+        <v>46102</v>
+      </c>
       <c r="F61" s="10"/>
-      <c r="G61" s="4"/>
+      <c r="G61" s="4" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A62" s="19" t="s">
@@ -2852,15 +2917,19 @@
         <v>46102</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E62" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E62" s="5">
+        <v>46102</v>
+      </c>
       <c r="F62" s="10"/>
-      <c r="G62" s="4"/>
+      <c r="G62" s="4" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A63" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>6</v>
@@ -2869,15 +2938,19 @@
         <v>46102</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E63" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E63" s="5">
+        <v>46102</v>
+      </c>
       <c r="F63" s="10"/>
-      <c r="G63" s="4"/>
+      <c r="G63" s="4" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A64" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>6</v>
@@ -2886,15 +2959,19 @@
         <v>46102</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E64" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E64" s="5">
+        <v>46103</v>
+      </c>
       <c r="F64" s="10"/>
-      <c r="G64" s="4"/>
+      <c r="G64" s="4" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A65" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>4</v>
@@ -2903,15 +2980,19 @@
         <v>46102</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E65" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E65" s="5">
+        <v>46102</v>
+      </c>
       <c r="F65" s="10"/>
-      <c r="G65" s="4"/>
+      <c r="G65" s="4" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>4</v>
@@ -2920,15 +3001,19 @@
         <v>46102</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E66" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E66" s="5">
+        <v>46102</v>
+      </c>
       <c r="F66" s="10"/>
-      <c r="G66" s="4"/>
+      <c r="G66" s="4" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A67" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>6</v>
@@ -2937,15 +3022,19 @@
         <v>46102</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E67" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E67" s="5">
+        <v>46103</v>
+      </c>
       <c r="F67" s="10"/>
-      <c r="G67" s="4"/>
+      <c r="G67" s="4" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>8</v>
@@ -2954,15 +3043,19 @@
         <v>46102</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E68" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E68" s="5">
+        <v>46103</v>
+      </c>
       <c r="F68" s="10"/>
-      <c r="G68" s="4"/>
+      <c r="G68" s="4" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69" s="19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>8</v>
@@ -2971,11 +3064,15 @@
         <v>46102</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E69" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="E69" s="5">
+        <v>46103</v>
+      </c>
       <c r="F69" s="10"/>
-      <c r="G69" s="4"/>
+      <c r="G69" s="4" t="s">
+        <v>99</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>